<commit_message>
feat: complete production-grade refactor with Decimal precision, key quarantine, typed field rules, CI, and expanded unit tests
</commit_message>
<xml_diff>
--- a/sample_data/bank_data.xlsx
+++ b/sample_data/bank_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,6 +590,114 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>INV-1007</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>$800.00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Zeta Enterprises</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>INV-1008</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>$950.00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Theta Co</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>INV-1008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>$950.00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Theta Co</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>INV-1010</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ERROR123</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Iota LLC</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>